<commit_message>
Leadlisten-Vorlage mit Erklärung und Branchen, Fundstelle je Betrieb
- Mustervorlage mit den Blättern Leadliste, Erklärung (Pflicht, Bedeutung,
  Format, Beispiel je Spalte, auch Prüfstufen) und Branchen
- Neue Spalte und neues Feld Fundstelle (URL) an der Organisation, im
  Import, im Formular, am Vorgang und in der Anrufliste
- docs/LEADLISTE_RECHERCHE.md: Ablauf und Anweisung für den Vertriebs-Chat

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import_vorlage.xlsx
+++ b/docs/import_vorlage.xlsx
@@ -2,12 +2,32 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rIdSheet1" state="visible"/>
+    <sheet name="Leadliste" sheetId="1" r:id="rIdSheet1" state="visible"/>
+    <sheet name="Erklärung" sheetId="2" r:id="rIdSheet2" state="visible"/>
+    <sheet name="Branchen" sheetId="3" r:id="rIdSheet3" state="visible"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Unknown</author>
+  </authors>
+  <commentList>    </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Unknown</author>
+  </authors>
+  <commentList>    </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Unknown</author>
@@ -23,19 +43,35 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="E8EEF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +85,12 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyBorder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle builtinId="0" name="Normal" xfId="0"/>
@@ -60,136 +100,141 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Z3"/>
   <sheetData>
-    <row r="1" spans="1:25" customHeight="0">
-      <c r="A1" s="0" t="inlineStr">
+    <row r="1" spans="1:26" customHeight="0">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Firmenname</t>
         </is>
       </c>
-      <c r="B1" s="0" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Rechtsform</t>
         </is>
       </c>
-      <c r="C1" s="0" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Branche</t>
         </is>
       </c>
-      <c r="D1" s="0" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>WZ-2008-Code</t>
         </is>
       </c>
-      <c r="E1" s="0" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Priorität</t>
         </is>
       </c>
-      <c r="F1" s="0" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Straße</t>
         </is>
       </c>
-      <c r="G1" s="0" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="H1" s="0" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ort</t>
         </is>
       </c>
-      <c r="I1" s="0" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Telefon</t>
         </is>
       </c>
-      <c r="J1" s="0" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>E-Mail</t>
         </is>
       </c>
-      <c r="K1" s="0" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="L1" s="0" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Fundstelle (URL)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Mitarbeitende</t>
         </is>
       </c>
-      <c r="M1" s="0" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Ausbildungsbetrieb</t>
         </is>
       </c>
-      <c r="N1" s="0" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Prüfstufe 1</t>
         </is>
       </c>
-      <c r="O1" s="0" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Prüfstufe 2</t>
         </is>
       </c>
-      <c r="P1" s="0" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Prüfstufe 3</t>
         </is>
       </c>
-      <c r="Q1" s="0" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Prüfstufe 4</t>
         </is>
       </c>
-      <c r="R1" s="0" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Prüfstufe 5</t>
         </is>
       </c>
-      <c r="S1" s="0" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Bemerkung Prüfung</t>
         </is>
       </c>
-      <c r="T1" s="0" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Anrede Ansprechpartner</t>
         </is>
       </c>
-      <c r="U1" s="0" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Vorname Ansprechpartner</t>
         </is>
       </c>
-      <c r="V1" s="0" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Nachname Ansprechpartner</t>
         </is>
       </c>
-      <c r="W1" s="0" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Funktion Ansprechpartner</t>
         </is>
       </c>
-      <c r="X1" s="0" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Telefon Ansprechpartner</t>
         </is>
       </c>
-      <c r="Y1" s="0" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>E-Mail Ansprechpartner</t>
         </is>
       </c>
     </row>
-    <row r="2" spans="1:25" customHeight="0">
+    <row r="2" spans="1:26" customHeight="0">
       <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Beispiel Steuerberatung GmbH</t>
@@ -247,71 +292,81 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
+          <t>https://www.beispiel-steuer.example/impressum</t>
+        </is>
+      </c>
+      <c r="M2" s="0" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="M2" s="0" t="inlineStr">
+      <c r="N2" s="0" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="N2" s="0" t="inlineStr">
+      <c r="O2" s="0" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O2" s="0" t="inlineStr">
+      <c r="P2" s="0" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="P2" s="0" t="inlineStr">
+      <c r="Q2" s="0" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="Q2" s="0" t="inlineStr">
-        <is>
-          <t>nein</t>
+      <c r="R2" s="0" t="inlineStr">
+        <is>
+          <t>ja</t>
         </is>
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="T2" s="0" t="inlineStr">
+        <is>
           <t>erfundene Beispielzeile</t>
         </is>
       </c>
-      <c r="T2" s="0" t="inlineStr">
+      <c r="U2" s="0" t="inlineStr">
         <is>
           <t>Frau</t>
         </is>
       </c>
-      <c r="U2" s="0" t="inlineStr">
+      <c r="V2" s="0" t="inlineStr">
         <is>
           <t>Erika</t>
         </is>
       </c>
-      <c r="V2" s="0" t="inlineStr">
+      <c r="W2" s="0" t="inlineStr">
         <is>
           <t>Mustermann</t>
         </is>
       </c>
-      <c r="W2" s="0" t="inlineStr">
+      <c r="X2" s="0" t="inlineStr">
         <is>
           <t>Geschäftsführung</t>
         </is>
       </c>
-      <c r="X2" s="0" t="inlineStr">
+      <c r="Y2" s="0" t="inlineStr">
         <is>
           <t>06131 000001</t>
         </is>
       </c>
-      <c r="Y2" s="0" t="inlineStr">
+      <c r="Z2" s="0" t="inlineStr">
         <is>
           <t>e.mustermann@beispiel-steuer.example</t>
         </is>
       </c>
     </row>
-    <row r="3" spans="1:25" customHeight="0">
+    <row r="3" spans="1:26" customHeight="0">
       <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Muster Logistik KG</t>
@@ -364,27 +419,944 @@
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
+          <t>https://www.muster-logistik.example/impressum</t>
+        </is>
+      </c>
+      <c r="M3" s="0" t="inlineStr">
+        <is>
           <t>45</t>
         </is>
       </c>
-      <c r="M3" s="0" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="O3" s="0" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="P3" s="0" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Q3" s="0" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="R3" s="0" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="S3" s="0" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <legacyDrawing r:id="rId_comments_vml1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E29"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="true"/>
+    <col min="2" max="2" width="12" customWidth="true"/>
+    <col min="3" max="3" width="60" customWidth="true"/>
+    <col min="4" max="4" width="36" customWidth="true"/>
+    <col min="5" max="5" width="36" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" customHeight="0">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Spalte</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Bedeutung</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Erlaubte Werte / Format</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Beispiel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:5" customHeight="0">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Firmenname</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Name des Betriebs wie im Impressum</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Muster Steuerberatung GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:5" customHeight="0">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Rechtsform</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Rechtsform des Betriebs</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>z. B. GmbH, UG (haftungsbeschränkt), e.K., GbR, KG, AG, PartG mbB</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:5" customHeight="0">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Branche</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Branche genau wie im Blatt „Branchen“ geschrieben</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Wert aus Blatt „Branchen“</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Steuerberatung</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:5" customHeight="0">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>WZ-2008-Code</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Branchenschlüssel des Statistischen Bundesamts. Leer lassen, wenn die Branche aus der Liste stammt, dann ergänzt das CRM den Code</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>z. B. 69.20</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>69.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:5" customHeight="0">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Priorität</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Wie gut passt der Betrieb? A = sehr gut, B = gut, C = möglich. Regeln siehe Rechercheanleitung</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>A, B oder C</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:5" customHeight="0">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Straße</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Straße und Hausnummer des Betriebs</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Musterstraße 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:5" customHeight="0">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>PLZ</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Postleitzahl. Wichtig für die Dublettenprüfung (Firmenname + PLZ)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>fünf Ziffern</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>55116</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:5" customHeight="0">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Ort des Betriebs</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Mainz</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:5" customHeight="0">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Telefon</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Zentrale Telefonnummer des Betriebs. Keine privaten Handynummern</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>wie auf der Website angegeben</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>06131 123456</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:5" customHeight="0">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>E-Mail</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Allgemeine E-Mail-Adresse des Betriebs</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>z. B. info@…</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>info@beispiel.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:5" customHeight="0">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Startseite des Betriebs</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Adresse mit https://</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.beispiel.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:5" customHeight="0">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Fundstelle (URL)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Genaue Seite, auf der die Angaben stehen, meist das Impressum. Nachweis, woher die Daten stammen</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Adresse mit https://</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.beispiel.de/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:5" customHeight="0">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Mitarbeitende</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Anzahl Mitarbeitende. Bei einer Spanne den unteren Wert. Leer lassen, wenn unbekannt</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ganze Zahl</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:5" customHeight="0">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildungsbetrieb</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Bildet der Betrieb aus (z. B. Ausbildungsplätze auf der Website oder bei der IHK)?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ja, nein oder leer</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O3" s="0" t="inlineStr">
+    </row>
+    <row r="16" spans="1:5" customHeight="0">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe 1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe: Bezeichnung laut Branchenmatrix ergänzen</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ja, nein oder leer (nicht geprüft)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="P3" s="0" t="inlineStr">
-        <is>
-          <t>nein</t>
+    </row>
+    <row r="17" spans="1:5" customHeight="0">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe 2</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe: Bezeichnung laut Branchenmatrix ergänzen</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ja, nein oder leer (nicht geprüft)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:5" customHeight="0">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe 3</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe: Bezeichnung laut Branchenmatrix ergänzen</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ja, nein oder leer (nicht geprüft)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:5" customHeight="0">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe 4</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe: Bezeichnung laut Branchenmatrix ergänzen</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>ja, nein oder leer (nicht geprüft)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:5" customHeight="0">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe 5</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Prüfstufe: Bezeichnung laut Branchenmatrix ergänzen</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>ja, nein oder leer (nicht geprüft)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:5" customHeight="0">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Bemerkung Prüfung</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>empfohlen</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Kurz: Warum könnte der Betrieb Bedarf an Weiterbildung haben? Auffälligkeiten</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Text, ein bis zwei Sätze</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>sucht laut Stellenanzeige Bürokraft, stellt Verwaltung auf digital um</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:5" customHeight="0">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Anrede Ansprechpartner</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Anrede der Ansprechperson</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Frau, Herr oder leer</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:5" customHeight="0">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Vorname Ansprechpartner</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Nur wenn öffentlich als geschäftliche Ansprechperson genannt, z. B. Geschäftsführung im Impressum</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Erika</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:5" customHeight="0">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Nachname Ansprechpartner</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Wie Vorname: nur öffentlich genannte geschäftliche Ansprechperson</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Mustermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:5" customHeight="0">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Funktion Ansprechpartner</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Funktion der Ansprechperson</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>z. B. Geschäftsführung, Personalleitung, Inhaber/in</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführung</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:5" customHeight="0">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Telefon Ansprechpartner</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Nur eine öffentlich genannte geschäftliche Durchwahl. Keine privaten Nummern</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>wie angegeben</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>06131 123457</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:5" customHeight="0">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>E-Mail Ansprechpartner</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Nur eine öffentlich genannte geschäftliche E-Mail-Adresse</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>E-Mail-Adresse</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>e.mustermann@beispiel.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:5" customHeight="0">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Quelle und Abrufdatum der ganzen Datei werden beim Import im CRM angegeben (Pflicht). Dubletten und Einträge der Sperrliste überspringt das CRM beim Import selbst.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <legacyDrawing r:id="rId_comments_vml1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="true"/>
+    <col min="2" max="2" width="16" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" customHeight="0">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Branche</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>WZ-2008-Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:2" customHeight="0">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Steuerberatung</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>69.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:2" customHeight="0">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Rechtsberatung</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>69.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:2" customHeight="0">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Architektur- und Ingenieurbüros</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>71.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:2" customHeight="0">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Immobilienmakler und -verwaltung</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>68.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:2" customHeight="0">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Versicherungsvermittlung</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>66.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:2" customHeight="0">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Unternehmensberatung</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:2" customHeight="0">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Werbung und Marketing</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>73.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:2" customHeight="0">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Elektroinstallation</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>43.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:2" customHeight="0">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Großhandel</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:2" customHeight="0">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Spedition und Logistik</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>52.29</t>
         </is>
       </c>
     </row>

</xml_diff>